<commit_message>
LSLS cant define Web LMS event
</commit_message>
<xml_diff>
--- a/2026_09_21/LSLS/report_for_BD_2026-09-22.xlsx
+++ b/2026_09_21/LSLS/report_for_BD_2026-09-22.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lenalee\work\2026_09\2026_09_21\LSLS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8643F3F5-6000-49C2-A837-A0C8179615FF}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E61DB595-1C44-4943-ADF9-52245B43D2B8}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="19560" windowHeight="12405" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -17,35 +17,47 @@
     <sheet name="foodwise eateries" sheetId="2" r:id="rId2"/>
     <sheet name="hase share function" sheetId="3" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="145621"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="14">
   <si>
     <t>Web</t>
-  </si>
-  <si>
-    <t>App</t>
-  </si>
-  <si>
-    <t>2026-08</t>
-  </si>
-  <si>
-    <t>少鹽少糖食店 icon impression</t>
-  </si>
-  <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>Mobile Web</t>
   </si>
   <si>
     <t>Android</t>
   </si>
   <si>
     <t>iOS</t>
+  </si>
+  <si>
+    <t>Date</t>
+  </si>
+  <si>
+    <t>App</t>
+  </si>
+  <si>
+    <r>
+      <t>少鹽少糖食店</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>SR1 page view</t>
+    </r>
+  </si>
+  <si>
+    <t>少鹽少糖食店 icon impression</t>
+  </si>
+  <si>
+    <t>Mobile Web</t>
   </si>
   <si>
     <t>咪嘥嘢食店 icon impression</t>
@@ -77,29 +89,11 @@
       <t>Daily Theme Listing Impressions (adv search)</t>
     </r>
   </si>
-  <si>
-    <r>
-      <t>少鹽少糖食店</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>SR1 page view</t>
-    </r>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
-  </numFmts>
   <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -141,16 +135,16 @@
     <font>
       <b/>
       <sz val="11"/>
-      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -194,15 +188,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="17" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="17" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -220,15 +214,16 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="17" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf numFmtId="17" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -575,9 +570,9 @@
     <col min="4" max="5" width="10.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -586,19 +581,13 @@
         <v>0</v>
       </c>
       <c r="C2" s="5" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="7">
-        <v>2565</v>
-      </c>
-      <c r="C3" s="8">
-        <v>6301</v>
-      </c>
+      <c r="A3" s="6"/>
+      <c r="B3" s="7"/>
+      <c r="C3" s="8"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -612,556 +601,246 @@
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="9" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="3"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" s="15">
-        <v>46235</v>
-      </c>
-      <c r="B8" s="12">
-        <v>20257</v>
-      </c>
-      <c r="C8" s="12">
-        <v>39493</v>
-      </c>
-      <c r="D8" s="12">
-        <v>87756</v>
-      </c>
-      <c r="E8" s="13">
-        <v>440460</v>
-      </c>
+      <c r="A8" s="11"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="14"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="15">
-        <v>46236</v>
-      </c>
-      <c r="B9" s="12">
-        <v>17623</v>
-      </c>
-      <c r="C9" s="12">
-        <v>36689</v>
-      </c>
-      <c r="D9" s="12">
-        <v>81841</v>
-      </c>
-      <c r="E9" s="13">
-        <v>417045</v>
-      </c>
+      <c r="A9" s="11"/>
+      <c r="B9" s="12"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="14"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" s="15">
-        <v>46237</v>
-      </c>
-      <c r="B10" s="12">
-        <v>44780</v>
-      </c>
-      <c r="C10" s="12">
-        <v>32543</v>
-      </c>
-      <c r="D10" s="12">
-        <v>64903</v>
-      </c>
-      <c r="E10" s="13">
-        <v>326647</v>
-      </c>
+      <c r="A10" s="11"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="14"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" s="15">
-        <v>46238</v>
-      </c>
-      <c r="B11" s="12">
-        <v>50576</v>
-      </c>
-      <c r="C11" s="12">
-        <v>34758</v>
-      </c>
-      <c r="D11" s="12">
-        <v>73025</v>
-      </c>
-      <c r="E11" s="13">
-        <v>363109</v>
-      </c>
+      <c r="A11" s="11"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="14"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" s="15">
-        <v>46239</v>
-      </c>
-      <c r="B12" s="12">
-        <v>50139</v>
-      </c>
-      <c r="C12" s="12">
-        <v>34689</v>
-      </c>
-      <c r="D12" s="12">
-        <v>74189</v>
-      </c>
-      <c r="E12" s="13">
-        <v>368825</v>
-      </c>
+      <c r="A12" s="11"/>
+      <c r="B12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="14"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" s="15">
-        <v>46240</v>
-      </c>
-      <c r="B13" s="12">
-        <v>51556</v>
-      </c>
-      <c r="C13" s="12">
-        <v>34699</v>
-      </c>
-      <c r="D13" s="12">
-        <v>76806</v>
-      </c>
-      <c r="E13" s="13">
-        <v>376998</v>
-      </c>
+      <c r="A13" s="11"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="14"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" s="15">
-        <v>46241</v>
-      </c>
-      <c r="B14" s="12">
-        <v>54856</v>
-      </c>
-      <c r="C14" s="12">
-        <v>37493</v>
-      </c>
-      <c r="D14" s="12">
-        <v>79905</v>
-      </c>
-      <c r="E14" s="13">
-        <v>403192</v>
-      </c>
+      <c r="A14" s="11"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="14"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" s="15">
-        <v>46242</v>
-      </c>
-      <c r="B15" s="12">
-        <v>30397</v>
-      </c>
-      <c r="C15" s="12">
-        <v>42042</v>
-      </c>
-      <c r="D15" s="12">
-        <v>90812</v>
-      </c>
-      <c r="E15" s="13">
-        <v>453735</v>
-      </c>
+      <c r="A15" s="11"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="14"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" s="15">
-        <v>46243</v>
-      </c>
-      <c r="B16" s="12">
-        <v>32759</v>
-      </c>
-      <c r="C16" s="12">
-        <v>37463</v>
-      </c>
-      <c r="D16" s="12">
-        <v>92661</v>
-      </c>
-      <c r="E16" s="13">
-        <v>460509</v>
-      </c>
+      <c r="A16" s="11"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="14"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" s="15">
-        <v>46244</v>
-      </c>
-      <c r="B17" s="12">
-        <v>55797</v>
-      </c>
-      <c r="C17" s="12">
-        <v>34911</v>
-      </c>
-      <c r="D17" s="12">
-        <v>71397</v>
-      </c>
-      <c r="E17" s="13">
-        <v>357474</v>
-      </c>
+      <c r="A17" s="11"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="14"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="15">
-        <v>46245</v>
-      </c>
-      <c r="B18" s="12">
-        <v>51840</v>
-      </c>
-      <c r="C18" s="12">
-        <v>36793</v>
-      </c>
-      <c r="D18" s="12">
-        <v>75184</v>
-      </c>
-      <c r="E18" s="13">
-        <v>373159</v>
-      </c>
+      <c r="A18" s="11"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="14"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" s="15">
-        <v>46246</v>
-      </c>
-      <c r="B19" s="12">
-        <v>49458</v>
-      </c>
-      <c r="C19" s="12">
-        <v>35953</v>
-      </c>
-      <c r="D19" s="12">
-        <v>73929</v>
-      </c>
-      <c r="E19" s="13">
-        <v>368155</v>
-      </c>
+      <c r="A19" s="11"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="14"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="15">
-        <v>46247</v>
-      </c>
-      <c r="B20" s="12">
-        <v>49973</v>
-      </c>
-      <c r="C20" s="12">
-        <v>35943</v>
-      </c>
-      <c r="D20" s="12">
-        <v>75886</v>
-      </c>
-      <c r="E20" s="13">
-        <v>378303</v>
-      </c>
+      <c r="A20" s="11"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="14"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="15">
-        <v>46248</v>
-      </c>
-      <c r="B21" s="12">
-        <v>49655</v>
-      </c>
-      <c r="C21" s="12">
-        <v>38266</v>
-      </c>
-      <c r="D21" s="12">
-        <v>77647</v>
-      </c>
-      <c r="E21" s="13">
-        <v>393146</v>
-      </c>
+      <c r="A21" s="11"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="14"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="15">
-        <v>46249</v>
-      </c>
-      <c r="B22" s="12">
-        <v>21250</v>
-      </c>
-      <c r="C22" s="12">
-        <v>42382</v>
-      </c>
-      <c r="D22" s="12">
-        <v>89846</v>
-      </c>
-      <c r="E22" s="13">
-        <v>453977</v>
-      </c>
+      <c r="A22" s="11"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="14"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="15">
-        <v>46250</v>
-      </c>
-      <c r="B23" s="12">
-        <v>18125</v>
-      </c>
-      <c r="C23" s="12">
-        <v>39811</v>
-      </c>
-      <c r="D23" s="12">
-        <v>87677</v>
-      </c>
-      <c r="E23" s="13">
-        <v>445441</v>
-      </c>
+      <c r="A23" s="11"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="14"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="15">
-        <v>46251</v>
-      </c>
-      <c r="B24" s="12">
-        <v>47037</v>
-      </c>
-      <c r="C24" s="12">
-        <v>34567</v>
-      </c>
-      <c r="D24" s="12">
-        <v>68206</v>
-      </c>
-      <c r="E24" s="13">
-        <v>345450</v>
-      </c>
+      <c r="A24" s="11"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="14"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A25" s="15">
-        <v>46252</v>
-      </c>
-      <c r="B25" s="12">
-        <v>48914</v>
-      </c>
-      <c r="C25" s="12">
-        <v>35848</v>
-      </c>
-      <c r="D25" s="12">
-        <v>73840</v>
-      </c>
-      <c r="E25" s="13">
-        <v>365220</v>
-      </c>
+      <c r="A25" s="11"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="14"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="15">
-        <v>46253</v>
-      </c>
-      <c r="B26" s="12">
-        <v>50218</v>
-      </c>
-      <c r="C26" s="12">
-        <v>35081</v>
-      </c>
-      <c r="D26" s="12">
-        <v>73921</v>
-      </c>
-      <c r="E26" s="13">
-        <v>371881</v>
-      </c>
+      <c r="A26" s="11"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="14"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A27" s="15">
-        <v>46254</v>
-      </c>
-      <c r="B27" s="12">
-        <v>48743</v>
-      </c>
-      <c r="C27" s="12">
-        <v>34957</v>
-      </c>
-      <c r="D27" s="12">
-        <v>72897</v>
-      </c>
-      <c r="E27" s="13">
-        <v>353294</v>
-      </c>
+      <c r="A27" s="11"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="14"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A28" s="15">
-        <v>46255</v>
-      </c>
-      <c r="B28" s="12">
-        <v>51547</v>
-      </c>
-      <c r="C28" s="12">
-        <v>36914</v>
-      </c>
-      <c r="D28" s="12">
-        <v>77213</v>
-      </c>
-      <c r="E28" s="13">
-        <v>394698</v>
-      </c>
+      <c r="A28" s="11"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="14"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A29" s="15">
-        <v>46256</v>
-      </c>
-      <c r="B29" s="12">
-        <v>22196</v>
-      </c>
-      <c r="C29" s="12">
-        <v>38402</v>
-      </c>
-      <c r="D29" s="12">
-        <v>88958</v>
-      </c>
-      <c r="E29" s="13">
-        <v>451576</v>
-      </c>
+      <c r="A29" s="11"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="14"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A30" s="15">
-        <v>46257</v>
-      </c>
-      <c r="B30" s="12">
-        <v>17203</v>
-      </c>
-      <c r="C30" s="12">
-        <v>37353</v>
-      </c>
-      <c r="D30" s="12">
-        <v>86341</v>
-      </c>
-      <c r="E30" s="13">
-        <v>429892</v>
-      </c>
+      <c r="A30" s="11"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="14"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A31" s="15">
-        <v>46258</v>
-      </c>
-      <c r="B31" s="12">
-        <v>44362</v>
-      </c>
-      <c r="C31" s="12">
-        <v>28271</v>
-      </c>
-      <c r="D31" s="12">
-        <v>67698</v>
-      </c>
-      <c r="E31" s="13">
-        <v>330782</v>
-      </c>
+      <c r="A31" s="11"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="14"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A32" s="15">
-        <v>46259</v>
-      </c>
-      <c r="B32" s="12">
-        <v>43385</v>
-      </c>
-      <c r="C32" s="12">
-        <v>27806</v>
-      </c>
-      <c r="D32" s="12">
-        <v>69149</v>
-      </c>
-      <c r="E32" s="13">
-        <v>340812</v>
-      </c>
+      <c r="A32" s="11"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="14"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="15">
-        <v>46260</v>
-      </c>
-      <c r="B33" s="12">
-        <v>44495</v>
-      </c>
-      <c r="C33" s="12">
-        <v>27222</v>
-      </c>
-      <c r="D33" s="12">
-        <v>67795</v>
-      </c>
-      <c r="E33" s="13">
-        <v>335798</v>
-      </c>
+      <c r="A33" s="11"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="14"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="15">
-        <v>46261</v>
-      </c>
-      <c r="B34" s="12">
-        <v>45524</v>
-      </c>
-      <c r="C34" s="12">
-        <v>30938</v>
-      </c>
-      <c r="D34" s="12">
-        <v>70094</v>
-      </c>
-      <c r="E34" s="13">
-        <v>339595</v>
-      </c>
+      <c r="A34" s="11"/>
+      <c r="B34" s="13"/>
+      <c r="C34" s="13"/>
+      <c r="D34" s="13"/>
+      <c r="E34" s="14"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="15">
-        <v>46262</v>
-      </c>
-      <c r="B35" s="12">
-        <v>48513</v>
-      </c>
-      <c r="C35" s="12">
-        <v>31571</v>
-      </c>
-      <c r="D35" s="12">
-        <v>80501</v>
-      </c>
-      <c r="E35" s="13">
-        <v>397097</v>
-      </c>
+      <c r="A35" s="11"/>
+      <c r="B35" s="13"/>
+      <c r="C35" s="13"/>
+      <c r="D35" s="13"/>
+      <c r="E35" s="14"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="15">
-        <v>46263</v>
-      </c>
-      <c r="B36" s="12">
-        <v>20694</v>
-      </c>
-      <c r="C36" s="12">
-        <v>36332</v>
-      </c>
-      <c r="D36" s="12">
-        <v>91961</v>
-      </c>
-      <c r="E36" s="13">
-        <v>455041</v>
-      </c>
+      <c r="A36" s="11"/>
+      <c r="B36" s="13"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="14"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="15">
-        <v>46264</v>
-      </c>
-      <c r="B37" s="12">
-        <v>18844</v>
-      </c>
-      <c r="C37" s="12">
-        <v>35628</v>
-      </c>
-      <c r="D37" s="12">
-        <v>88471</v>
-      </c>
-      <c r="E37" s="13">
-        <v>438080</v>
-      </c>
+      <c r="A37" s="11"/>
+      <c r="B37" s="13"/>
+      <c r="C37" s="13"/>
+      <c r="D37" s="13"/>
+      <c r="E37" s="14"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="15">
-        <v>46265</v>
-      </c>
-      <c r="B38" s="12">
-        <v>40599</v>
-      </c>
-      <c r="C38" s="12">
-        <v>28041</v>
-      </c>
-      <c r="D38" s="12">
-        <v>61609</v>
-      </c>
-      <c r="E38" s="13">
-        <v>309798</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="11"/>
+      <c r="B38" s="13"/>
+      <c r="C38" s="13"/>
+      <c r="D38" s="13"/>
+      <c r="E38" s="15"/>
+    </row>
+    <row r="41" spans="1:5" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
         <v>13</v>
       </c>
@@ -1172,19 +851,13 @@
         <v>0</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="6" t="s">
-        <v>2</v>
-      </c>
-      <c r="B43" s="7">
-        <v>0</v>
-      </c>
-      <c r="C43" s="8">
-        <v>543</v>
-      </c>
+      <c r="A43" s="6"/>
+      <c r="B43" s="7"/>
+      <c r="C43" s="8"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1209,237 +882,237 @@
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B2" s="10" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="11"/>
       <c r="B3" s="12"/>
-      <c r="C3" s="12"/>
-      <c r="D3" s="12"/>
-      <c r="E3" s="13"/>
+      <c r="C3" s="13"/>
+      <c r="D3" s="13"/>
+      <c r="E3" s="14"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="11"/>
       <c r="B4" s="12"/>
-      <c r="C4" s="12"/>
-      <c r="D4" s="12"/>
-      <c r="E4" s="13"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="13"/>
+      <c r="E4" s="14"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="11"/>
       <c r="B5" s="12"/>
-      <c r="C5" s="12"/>
-      <c r="D5" s="12"/>
-      <c r="E5" s="13"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="14"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" s="11"/>
-      <c r="B6" s="12"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="12"/>
-      <c r="E6" s="13"/>
+      <c r="B6" s="13"/>
+      <c r="C6" s="13"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="14"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" s="11"/>
-      <c r="B7" s="12"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="12"/>
-      <c r="E7" s="13"/>
+      <c r="B7" s="13"/>
+      <c r="C7" s="13"/>
+      <c r="D7" s="13"/>
+      <c r="E7" s="14"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" s="11"/>
       <c r="B8" s="12"/>
-      <c r="C8" s="12"/>
-      <c r="D8" s="12"/>
-      <c r="E8" s="13"/>
+      <c r="C8" s="13"/>
+      <c r="D8" s="13"/>
+      <c r="E8" s="14"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" s="11"/>
       <c r="B9" s="12"/>
-      <c r="C9" s="12"/>
-      <c r="D9" s="12"/>
-      <c r="E9" s="13"/>
+      <c r="C9" s="13"/>
+      <c r="D9" s="13"/>
+      <c r="E9" s="14"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" s="11"/>
       <c r="B10" s="12"/>
-      <c r="C10" s="12"/>
-      <c r="D10" s="12"/>
-      <c r="E10" s="13"/>
+      <c r="C10" s="13"/>
+      <c r="D10" s="13"/>
+      <c r="E10" s="14"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" s="11"/>
       <c r="B11" s="12"/>
-      <c r="C11" s="12"/>
-      <c r="D11" s="12"/>
-      <c r="E11" s="13"/>
+      <c r="C11" s="13"/>
+      <c r="D11" s="13"/>
+      <c r="E11" s="14"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" s="11"/>
       <c r="B12" s="12"/>
-      <c r="C12" s="12"/>
-      <c r="D12" s="12"/>
-      <c r="E12" s="13"/>
+      <c r="C12" s="13"/>
+      <c r="D12" s="13"/>
+      <c r="E12" s="14"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" s="11"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="13"/>
+      <c r="B13" s="13"/>
+      <c r="C13" s="13"/>
+      <c r="D13" s="13"/>
+      <c r="E13" s="14"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" s="11"/>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="13"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+      <c r="D14" s="13"/>
+      <c r="E14" s="14"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" s="11"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="13"/>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="14"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="11"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="13"/>
+      <c r="B16" s="13"/>
+      <c r="C16" s="13"/>
+      <c r="D16" s="13"/>
+      <c r="E16" s="14"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="11"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="13"/>
+      <c r="B17" s="13"/>
+      <c r="C17" s="13"/>
+      <c r="D17" s="13"/>
+      <c r="E17" s="14"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="11"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="13"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13"/>
+      <c r="D18" s="13"/>
+      <c r="E18" s="14"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="11"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="13"/>
+      <c r="B19" s="13"/>
+      <c r="C19" s="13"/>
+      <c r="D19" s="13"/>
+      <c r="E19" s="14"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="11"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="13"/>
+      <c r="B20" s="13"/>
+      <c r="C20" s="13"/>
+      <c r="D20" s="13"/>
+      <c r="E20" s="14"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="11"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="13"/>
+      <c r="B21" s="13"/>
+      <c r="C21" s="13"/>
+      <c r="D21" s="13"/>
+      <c r="E21" s="14"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="11"/>
-      <c r="B22" s="12"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="13"/>
+      <c r="B22" s="13"/>
+      <c r="C22" s="13"/>
+      <c r="D22" s="13"/>
+      <c r="E22" s="14"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="11"/>
-      <c r="B23" s="12"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="13"/>
+      <c r="B23" s="13"/>
+      <c r="C23" s="13"/>
+      <c r="D23" s="13"/>
+      <c r="E23" s="14"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="11"/>
-      <c r="B24" s="12"/>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="13"/>
+      <c r="B24" s="13"/>
+      <c r="C24" s="13"/>
+      <c r="D24" s="13"/>
+      <c r="E24" s="14"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="11"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="13"/>
+      <c r="B25" s="13"/>
+      <c r="C25" s="13"/>
+      <c r="D25" s="13"/>
+      <c r="E25" s="14"/>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="11"/>
-      <c r="B26" s="12"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="13"/>
+      <c r="B26" s="13"/>
+      <c r="C26" s="13"/>
+      <c r="D26" s="13"/>
+      <c r="E26" s="14"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="11"/>
-      <c r="B27" s="12"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="13"/>
+      <c r="B27" s="13"/>
+      <c r="C27" s="13"/>
+      <c r="D27" s="13"/>
+      <c r="E27" s="14"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="11"/>
-      <c r="B28" s="12"/>
-      <c r="C28" s="12"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="13"/>
+      <c r="B28" s="13"/>
+      <c r="C28" s="13"/>
+      <c r="D28" s="13"/>
+      <c r="E28" s="14"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="11"/>
-      <c r="B29" s="12"/>
-      <c r="C29" s="12"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="13"/>
+      <c r="B29" s="13"/>
+      <c r="C29" s="13"/>
+      <c r="D29" s="13"/>
+      <c r="E29" s="14"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="11"/>
-      <c r="B30" s="12"/>
-      <c r="C30" s="12"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="13"/>
+      <c r="B30" s="13"/>
+      <c r="C30" s="13"/>
+      <c r="D30" s="13"/>
+      <c r="E30" s="14"/>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="11"/>
-      <c r="B31" s="12"/>
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="13"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13"/>
+      <c r="D31" s="13"/>
+      <c r="E31" s="14"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="11"/>
-      <c r="B32" s="12"/>
-      <c r="C32" s="12"/>
-      <c r="D32" s="12"/>
-      <c r="E32" s="13"/>
+      <c r="B32" s="13"/>
+      <c r="C32" s="13"/>
+      <c r="D32" s="13"/>
+      <c r="E32" s="14"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" s="11"/>
-      <c r="B33" s="12"/>
-      <c r="C33" s="12"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="13"/>
+      <c r="B33" s="13"/>
+      <c r="C33" s="13"/>
+      <c r="D33" s="13"/>
+      <c r="E33" s="15"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1468,193 +1141,193 @@
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" s="14"/>
+      <c r="A2" s="16"/>
       <c r="B2" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" s="14"/>
+      <c r="A3" s="16"/>
       <c r="B3" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" s="14"/>
+      <c r="A4" s="16"/>
       <c r="B4" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" s="14"/>
+      <c r="A5" s="16"/>
       <c r="B5" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" s="14"/>
+      <c r="A6" s="16"/>
       <c r="B6" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" s="14"/>
+      <c r="A7" s="16"/>
       <c r="B7" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" s="14"/>
+      <c r="A8" s="16"/>
       <c r="B8" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" s="14"/>
+      <c r="A9" s="16"/>
       <c r="B9" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" s="14"/>
+      <c r="A10" s="16"/>
       <c r="B10" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" s="14"/>
+      <c r="A11" s="16"/>
       <c r="B11" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" s="14"/>
+      <c r="A12" s="16"/>
       <c r="B12" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" s="14"/>
+      <c r="A13" s="16"/>
       <c r="B13" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" s="14"/>
+      <c r="A14" s="16"/>
       <c r="B14" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" s="14"/>
+      <c r="A15" s="16"/>
       <c r="B15" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" s="14"/>
+      <c r="A16" s="16"/>
       <c r="B16" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A17" s="14"/>
+      <c r="A17" s="16"/>
       <c r="B17" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A18" s="14"/>
+      <c r="A18" s="16"/>
       <c r="B18" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A19" s="14"/>
+      <c r="A19" s="16"/>
       <c r="B19" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A20" s="14"/>
+      <c r="A20" s="16"/>
       <c r="B20" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A21" s="14"/>
+      <c r="A21" s="16"/>
       <c r="B21" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="14"/>
+      <c r="A22" s="16"/>
       <c r="B22" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="14"/>
+      <c r="A23" s="16"/>
       <c r="B23" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="14"/>
+      <c r="A24" s="16"/>
       <c r="B24" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A25" s="14"/>
+      <c r="A25" s="16"/>
       <c r="B25" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A26" s="14"/>
+      <c r="A26" s="16"/>
       <c r="B26" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A27" s="14"/>
+      <c r="A27" s="16"/>
       <c r="B27" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A28" s="14"/>
+      <c r="A28" s="16"/>
       <c r="B28" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A29" s="14"/>
+      <c r="A29" s="16"/>
       <c r="B29" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A30" s="14"/>
+      <c r="A30" s="16"/>
       <c r="B30" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A31" s="14"/>
+      <c r="A31" s="16"/>
       <c r="B31" t="s">
         <v>12</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A32" s="14"/>
+      <c r="A32" s="16"/>
       <c r="B32" t="s">
         <v>12</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>